<commit_message>
feat: court search supports party name input on ssgo
</commit_message>
<xml_diff>
--- a/court-search/input.xlsx
+++ b/court-search/input.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -471,6 +471,11 @@
           <t>비고</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>당사자명</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -488,6 +493,11 @@
           <t>인도명령</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>주택</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -505,6 +515,11 @@
           <t>인도명령</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>주택</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -522,6 +537,11 @@
           <t>인도명령</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>주택</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -539,6 +559,11 @@
           <t>인도명령</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>주택</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -554,6 +579,11 @@
       <c r="C6" s="2" t="inlineStr">
         <is>
           <t>인도명령</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>주택</t>
         </is>
       </c>
     </row>

</xml_diff>